<commit_message>
Practiced Textjoin, TextSplit, Find and MID functions
</commit_message>
<xml_diff>
--- a/2_Formulas_Functions/8_Text_Functions.xlsx
+++ b/2_Formulas_Functions/8_Text_Functions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10511"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\Developer\_Courses\Excel\Excel_Data_Analytics_Course\2_Formulas_Functions\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dan/Desktop/data-analytics/Excel_Data_Analytics_Course/2_Formulas_Functions/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289F5FEB-D4A0-4E30-9E0C-8AA9F558B1FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C76D0F2-034F-7748-960E-55AC26E38706}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2205" yWindow="2205" windowWidth="21600" windowHeight="11993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="500" yWindow="920" windowWidth="30080" windowHeight="19280" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="8" r:id="rId1"/>
@@ -19,6 +19,12 @@
     <sheet name="Text_Search" sheetId="11" r:id="rId4"/>
     <sheet name="Skills" sheetId="12" r:id="rId5"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlchart.v1.0" hidden="1">Skills!$A$35:$A$50</definedName>
+    <definedName name="_xlchart.v1.1" hidden="1">Skills!$B$35:$B$50</definedName>
+    <definedName name="_xlchart.v2.2" hidden="1">Skills!$A$35:$A$50</definedName>
+    <definedName name="_xlchart.v2.3" hidden="1">Skills!$B$35:$B$50</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -40,7 +46,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -566,7 +572,7 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
-  <c:lang val="en-US"/>
+  <c:lang val="en-GB"/>
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
@@ -935,7 +941,434 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-GB"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-GB"/>
+              <a:t>Top Skills by Job</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-GB" baseline="0"/>
+              <a:t> Applicants</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-GB"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout>
+        <c:manualLayout>
+          <c:layoutTarget val="inner"/>
+          <c:xMode val="edge"/>
+          <c:yMode val="edge"/>
+          <c:x val="0.12057181982686947"/>
+          <c:y val="0.15115846298472918"/>
+          <c:w val="0.82834743483151563"/>
+          <c:h val="0.78350781075892595"/>
+        </c:manualLayout>
+      </c:layout>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:strRef>
+              <c:f>Skills!$A$35:$A$50</c:f>
+              <c:strCache>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>Kafka</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>DataBricks</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Spark</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Python</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>GCP</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Power BI</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Airflow</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Hadoop</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>R</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Azure</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>Java</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>SQL</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>Snowflake</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>Scala</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>Excel</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>Tableau</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Skills!$B$35:$B$50</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="16"/>
+                <c:pt idx="0">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>7</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>4</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>2</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-320B-394F-AC28-2E1DD0800F0C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="182"/>
+        <c:axId val="432706191"/>
+        <c:axId val="432707903"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="432706191"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="432707903"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="432707903"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="432706191"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -1480,6 +1913,511 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="216">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
@@ -1513,6 +2451,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>635000</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>328084</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>116417</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{51313692-1948-A79F-7C3F-FE411B0F18CC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1785,27 +2759,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B5E7F13-C613-4452-9CDB-2C26D6876D9D}">
   <dimension ref="A1:V21"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="17.59765625" customWidth="1"/>
-    <col min="2" max="2" width="14.265625" customWidth="1"/>
-    <col min="3" max="3" width="27.265625" customWidth="1"/>
-    <col min="4" max="4" width="17.59765625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="26.265625" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="2" max="2" width="14.33203125" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="26.33203125" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="22" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="8.86328125" customWidth="1"/>
-    <col min="10" max="10" width="34.73046875" customWidth="1"/>
-    <col min="11" max="11" width="8.86328125" customWidth="1"/>
+    <col min="9" max="9" width="8.83203125" customWidth="1"/>
+    <col min="10" max="10" width="34.6640625" customWidth="1"/>
+    <col min="11" max="11" width="8.83203125" customWidth="1"/>
     <col min="12" max="12" width="13.33203125" customWidth="1"/>
-    <col min="13" max="13" width="15.46484375" customWidth="1"/>
-    <col min="14" max="14" width="8.86328125" customWidth="1"/>
-    <col min="15" max="15" width="16.3984375" customWidth="1"/>
+    <col min="13" max="13" width="15.5" customWidth="1"/>
+    <col min="14" max="14" width="8.83203125" customWidth="1"/>
+    <col min="15" max="15" width="16.33203125" customWidth="1"/>
     <col min="17" max="19" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
@@ -1853,7 +2827,7 @@
       <c r="U1" s="17"/>
       <c r="V1" s="17"/>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>72</v>
       </c>
@@ -1877,6 +2851,21 @@
       </c>
       <c r="H2" s="6" t="s">
         <v>11</v>
+      </c>
+      <c r="J2" t="str">
+        <f>_xlfn.TEXTJOIN(" ", TRUE,F2:G2)</f>
+        <v>457 Oak St San Jose, CA, 95101</v>
+      </c>
+      <c r="L2" t="str" cm="1">
+        <f t="array" ref="L2:M2">_xlfn.TEXTSPLIT(B2," ")</f>
+        <v>Pam</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Beesly</v>
+      </c>
+      <c r="O2" t="str">
+        <f>RIGHT(A2,7)</f>
+        <v>0123548</v>
       </c>
       <c r="Q2">
         <f>FIND(",", G2)+LEN(", ")</f>
@@ -1890,8 +2879,20 @@
         <f>MID(G2,Q2,R2-Q2)</f>
         <v>CA</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T2">
+        <f>FIND(",",G2)+LEN(", ")</f>
+        <v>11</v>
+      </c>
+      <c r="U2">
+        <f>FIND(",",G2,T2)</f>
+        <v>13</v>
+      </c>
+      <c r="V2" t="str">
+        <f>MID(G2,T2,U2-T2)</f>
+        <v>CA</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>71</v>
       </c>
@@ -1916,20 +2917,47 @@
       <c r="H3" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="J3" t="str">
+        <f t="shared" ref="J3:J21" si="0">_xlfn.TEXTJOIN(" ", TRUE,F3:G3)</f>
+        <v>203 Birch St Chicago, IL, 60601</v>
+      </c>
+      <c r="L3" t="str" cm="1">
+        <f t="array" ref="L3:M3">_xlfn.TEXTSPLIT(B3," ")</f>
+        <v>Michael</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Scott</v>
+      </c>
+      <c r="O3" t="str">
+        <f t="shared" ref="O3:O21" si="1">RIGHT(A3,7)</f>
+        <v>0123549</v>
+      </c>
       <c r="Q3">
-        <f t="shared" ref="Q3:Q21" si="0">FIND(",", G3)+LEN(", ")</f>
+        <f t="shared" ref="Q3:Q21" si="2">FIND(",", G3)+LEN(", ")</f>
         <v>10</v>
       </c>
       <c r="R3">
-        <f t="shared" ref="R3:R21" si="1">FIND(",",G3,Q3)</f>
+        <f t="shared" ref="R3:R21" si="3">FIND(",",G3,Q3)</f>
         <v>12</v>
       </c>
       <c r="S3" t="str">
-        <f t="shared" ref="S3:S21" si="2">MID(G3,Q3,R3-Q3)</f>
+        <f t="shared" ref="S3:S21" si="4">MID(G3,Q3,R3-Q3)</f>
         <v>IL</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T3">
+        <f t="shared" ref="T3:T21" si="5">FIND(",",G3)+LEN(", ")</f>
+        <v>10</v>
+      </c>
+      <c r="U3">
+        <f t="shared" ref="U3:U21" si="6">FIND(",",G3,T3)</f>
+        <v>12</v>
+      </c>
+      <c r="V3" t="str">
+        <f t="shared" ref="V3:V21" si="7">MID(G3,T3,U3-T3)</f>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>73</v>
       </c>
@@ -1954,20 +2982,47 @@
       <c r="H4" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="J4" t="str">
+        <f t="shared" si="0"/>
+        <v>790 Pine St Chicago, IL, 60601</v>
+      </c>
+      <c r="L4" t="str" cm="1">
+        <f t="array" ref="L4:M4">_xlfn.TEXTSPLIT(B4," ")</f>
+        <v>Kevin</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Malone</v>
+      </c>
+      <c r="O4" t="str">
+        <f t="shared" si="1"/>
+        <v>0123550</v>
+      </c>
       <c r="Q4">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R4">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S4" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T4">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U4">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V4" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>74</v>
       </c>
@@ -1992,20 +3047,47 @@
       <c r="H5" s="6" t="s">
         <v>11</v>
       </c>
+      <c r="J5" t="str">
+        <f t="shared" si="0"/>
+        <v>457 Oak St San Jose, CA, 95101</v>
+      </c>
+      <c r="L5" t="str" cm="1">
+        <f t="array" ref="L5:M5">_xlfn.TEXTSPLIT(B5," ")</f>
+        <v>Pam</v>
+      </c>
+      <c r="M5" t="str">
+        <v>Beesly</v>
+      </c>
+      <c r="O5" t="str">
+        <f t="shared" si="1"/>
+        <v>0123551</v>
+      </c>
       <c r="Q5">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="R5">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="S5" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>CA</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T5">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="U5">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="V5" t="str">
+        <f t="shared" si="7"/>
+        <v>CA</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>75</v>
       </c>
@@ -2030,20 +3112,47 @@
       <c r="H6" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="J6" t="str">
+        <f t="shared" si="0"/>
+        <v>459 Oak St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L6" t="str" cm="1">
+        <f t="array" ref="L6:M6">_xlfn.TEXTSPLIT(B6," ")</f>
+        <v>Jim</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Halpert</v>
+      </c>
+      <c r="O6" t="str">
+        <f t="shared" si="1"/>
+        <v>0123552</v>
+      </c>
       <c r="Q6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R6">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S6" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T6">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V6" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>76</v>
       </c>
@@ -2068,20 +3177,47 @@
       <c r="H7" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="J7" t="str">
+        <f t="shared" si="0"/>
+        <v>204 Birch St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L7" t="str" cm="1">
+        <f t="array" ref="L7:M7">_xlfn.TEXTSPLIT(B7," ")</f>
+        <v>Ryan</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Howard</v>
+      </c>
+      <c r="O7" t="str">
+        <f t="shared" si="1"/>
+        <v>0123553</v>
+      </c>
       <c r="Q7">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S7" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T7">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V7" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>77</v>
       </c>
@@ -2106,20 +3242,47 @@
       <c r="H8" s="6" t="s">
         <v>6</v>
       </c>
+      <c r="J8" t="str">
+        <f t="shared" si="0"/>
+        <v>790 Pine St Chicago, IL, 60601</v>
+      </c>
+      <c r="L8" t="str" cm="1">
+        <f t="array" ref="L8:M8">_xlfn.TEXTSPLIT(B8," ")</f>
+        <v>Kevin</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Malone</v>
+      </c>
+      <c r="O8" t="str">
+        <f t="shared" si="1"/>
+        <v>0123554</v>
+      </c>
       <c r="Q8">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R8">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S8" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T8">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V8" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>78</v>
       </c>
@@ -2144,20 +3307,47 @@
       <c r="H9" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="J9" t="str">
+        <f t="shared" si="0"/>
+        <v>204 Birch St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L9" t="str" cm="1">
+        <f t="array" ref="L9:M9">_xlfn.TEXTSPLIT(B9," ")</f>
+        <v>Ryan</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Howard</v>
+      </c>
+      <c r="O9" t="str">
+        <f t="shared" si="1"/>
+        <v>0123555</v>
+      </c>
       <c r="Q9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R9">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S9" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T9">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V9" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>79</v>
       </c>
@@ -2182,20 +3372,47 @@
       <c r="H10" s="6" t="s">
         <v>18</v>
       </c>
+      <c r="J10" t="str">
+        <f t="shared" si="0"/>
+        <v>123 Elm St Chicago, IL, 60601</v>
+      </c>
+      <c r="L10" t="str" cm="1">
+        <f t="array" ref="L10:M10">_xlfn.TEXTSPLIT(B10," ")</f>
+        <v>Stanley</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Hudson</v>
+      </c>
+      <c r="O10" t="str">
+        <f t="shared" si="1"/>
+        <v>0123556</v>
+      </c>
       <c r="Q10">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R10">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S10" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T10">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V10" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>80</v>
       </c>
@@ -2220,20 +3437,47 @@
       <c r="H11" s="6" t="s">
         <v>13</v>
       </c>
+      <c r="J11" t="str">
+        <f t="shared" si="0"/>
+        <v>123 Elm St Los Angeles, CA, 90001</v>
+      </c>
+      <c r="L11" t="str" cm="1">
+        <f t="array" ref="L11:M11">_xlfn.TEXTSPLIT(B11," ")</f>
+        <v>Angela</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Martin</v>
+      </c>
+      <c r="O11" t="str">
+        <f t="shared" si="1"/>
+        <v>0123557</v>
+      </c>
       <c r="Q11">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>14</v>
       </c>
       <c r="R11">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="S11" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>CA</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T11">
+        <f t="shared" si="5"/>
+        <v>14</v>
+      </c>
+      <c r="U11">
+        <f t="shared" si="6"/>
+        <v>16</v>
+      </c>
+      <c r="V11" t="str">
+        <f t="shared" si="7"/>
+        <v>CA</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>81</v>
       </c>
@@ -2258,20 +3502,47 @@
       <c r="H12" s="6" t="s">
         <v>17</v>
       </c>
+      <c r="J12" t="str">
+        <f t="shared" si="0"/>
+        <v>123 Elm St San Diego, CA, 92101</v>
+      </c>
+      <c r="L12" t="str" cm="1">
+        <f t="array" ref="L12:M12">_xlfn.TEXTSPLIT(B12," ")</f>
+        <v>Dwight</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Schrute</v>
+      </c>
+      <c r="O12" t="str">
+        <f t="shared" si="1"/>
+        <v>0123558</v>
+      </c>
       <c r="Q12">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="R12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="S12" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>CA</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T12">
+        <f t="shared" si="5"/>
+        <v>12</v>
+      </c>
+      <c r="U12">
+        <f t="shared" si="6"/>
+        <v>14</v>
+      </c>
+      <c r="V12" t="str">
+        <f t="shared" si="7"/>
+        <v>CA</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
@@ -2296,20 +3567,47 @@
       <c r="H13" s="6" t="s">
         <v>16</v>
       </c>
+      <c r="J13" t="str">
+        <f t="shared" si="0"/>
+        <v>202 Birch St Chicago, IL, 60601</v>
+      </c>
+      <c r="L13" t="str" cm="1">
+        <f t="array" ref="L13:M13">_xlfn.TEXTSPLIT(B13," ")</f>
+        <v>Oscar</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Martinez</v>
+      </c>
+      <c r="O13" t="str">
+        <f t="shared" si="1"/>
+        <v>0123559</v>
+      </c>
       <c r="Q13">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S13" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T13">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U13">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V13" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>83</v>
       </c>
@@ -2334,20 +3632,47 @@
       <c r="H14" s="6" t="s">
         <v>15</v>
       </c>
+      <c r="J14" t="str">
+        <f t="shared" si="0"/>
+        <v>204 Birch St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L14" t="str" cm="1">
+        <f t="array" ref="L14:M14">_xlfn.TEXTSPLIT(B14," ")</f>
+        <v>Ryan</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Howard</v>
+      </c>
+      <c r="O14" t="str">
+        <f t="shared" si="1"/>
+        <v>0123560</v>
+      </c>
       <c r="Q14">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S14" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T14">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U14">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V14" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>84</v>
       </c>
@@ -2372,20 +3697,47 @@
       <c r="H15" s="6" t="s">
         <v>19</v>
       </c>
+      <c r="J15" t="str">
+        <f t="shared" si="0"/>
+        <v>123 Elm St Chicago, IL, 60601</v>
+      </c>
+      <c r="L15" t="str" cm="1">
+        <f t="array" ref="L15:M15">_xlfn.TEXTSPLIT(B15," ")</f>
+        <v>Phyllis</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Vance</v>
+      </c>
+      <c r="O15" t="str">
+        <f t="shared" si="1"/>
+        <v>0123561</v>
+      </c>
       <c r="Q15">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S15" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.45">
+      <c r="T15">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U15">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V15" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>85</v>
       </c>
@@ -2410,20 +3762,47 @@
       <c r="H16" s="6" t="s">
         <v>20</v>
       </c>
+      <c r="J16" t="str">
+        <f t="shared" si="0"/>
+        <v>456 Oak St Chicago, IL, 60601</v>
+      </c>
+      <c r="L16" t="str" cm="1">
+        <f t="array" ref="L16:M16">_xlfn.TEXTSPLIT(B16," ")</f>
+        <v>Meredith</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Palmer</v>
+      </c>
+      <c r="O16" t="str">
+        <f t="shared" si="1"/>
+        <v>0123562</v>
+      </c>
       <c r="Q16">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S16" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="T16">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U16">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V16" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>86</v>
       </c>
@@ -2448,20 +3827,47 @@
       <c r="H17" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="J17" t="str">
+        <f t="shared" si="0"/>
+        <v>203 Birch St Chicago, IL, 60602</v>
+      </c>
+      <c r="L17" t="str" cm="1">
+        <f t="array" ref="L17:M17">_xlfn.TEXTSPLIT(B17," ")</f>
+        <v>Michael</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Scott</v>
+      </c>
+      <c r="O17" t="str">
+        <f t="shared" si="1"/>
+        <v>0123563</v>
+      </c>
       <c r="Q17">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="R17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
       <c r="S17" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>IL</v>
       </c>
-    </row>
-    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="T17">
+        <f t="shared" si="5"/>
+        <v>10</v>
+      </c>
+      <c r="U17">
+        <f t="shared" si="6"/>
+        <v>12</v>
+      </c>
+      <c r="V17" t="str">
+        <f t="shared" si="7"/>
+        <v>IL</v>
+      </c>
+    </row>
+    <row r="18" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>87</v>
       </c>
@@ -2486,20 +3892,47 @@
       <c r="H18" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="J18" t="str">
+        <f t="shared" si="0"/>
+        <v>459 Oak St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L18" t="str" cm="1">
+        <f t="array" ref="L18:M18">_xlfn.TEXTSPLIT(B18," ")</f>
+        <v>Jim</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Halpert</v>
+      </c>
+      <c r="O18" t="str">
+        <f t="shared" si="1"/>
+        <v>0123564</v>
+      </c>
       <c r="Q18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S18" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="T18">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U18">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V18" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
@@ -2524,20 +3957,47 @@
       <c r="H19" s="6" t="s">
         <v>8</v>
       </c>
+      <c r="J19" t="str">
+        <f t="shared" si="0"/>
+        <v>456 Oak St New York, NY, 10001</v>
+      </c>
+      <c r="L19" t="str" cm="1">
+        <f t="array" ref="L19:M19">_xlfn.TEXTSPLIT(B19," ")</f>
+        <v>Kelly</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Kapoor</v>
+      </c>
+      <c r="O19" t="str">
+        <f t="shared" si="1"/>
+        <v>0123565</v>
+      </c>
       <c r="Q19">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="R19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="S19" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>NY</v>
       </c>
-    </row>
-    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="T19">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="U19">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="V19" t="str">
+        <f t="shared" si="7"/>
+        <v>NY</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>89</v>
       </c>
@@ -2562,20 +4022,47 @@
       <c r="H20" s="6" t="s">
         <v>10</v>
       </c>
+      <c r="J20" t="str">
+        <f t="shared" si="0"/>
+        <v>459 Oak St Philadelphia, PA, 19101</v>
+      </c>
+      <c r="L20" t="str" cm="1">
+        <f t="array" ref="L20:M20">_xlfn.TEXTSPLIT(B20," ")</f>
+        <v>Jim</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Halpert</v>
+      </c>
+      <c r="O20" t="str">
+        <f t="shared" si="1"/>
+        <v>0123566</v>
+      </c>
       <c r="Q20">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>15</v>
       </c>
       <c r="R20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="S20" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>PA</v>
       </c>
-    </row>
-    <row r="21" spans="1:19" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="T20">
+        <f t="shared" si="5"/>
+        <v>15</v>
+      </c>
+      <c r="U20">
+        <f t="shared" si="6"/>
+        <v>17</v>
+      </c>
+      <c r="V20" t="str">
+        <f t="shared" si="7"/>
+        <v>PA</v>
+      </c>
+    </row>
+    <row r="21" spans="1:22" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>90</v>
       </c>
@@ -2600,16 +4087,43 @@
       <c r="H21" s="8" t="s">
         <v>10</v>
       </c>
+      <c r="J21" t="str">
+        <f t="shared" si="0"/>
+        <v>459 Oak St New York, NY, 10001</v>
+      </c>
+      <c r="L21" t="str" cm="1">
+        <f t="array" ref="L21:M21">_xlfn.TEXTSPLIT(B21," ")</f>
+        <v>Jim</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Halpert</v>
+      </c>
+      <c r="O21" t="str">
+        <f t="shared" si="1"/>
+        <v>0123567</v>
+      </c>
       <c r="Q21">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>11</v>
       </c>
       <c r="R21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="S21" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
+        <v>NY</v>
+      </c>
+      <c r="T21">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="U21">
+        <f t="shared" si="6"/>
+        <v>13</v>
+      </c>
+      <c r="V21" t="str">
+        <f t="shared" si="7"/>
         <v>NY</v>
       </c>
     </row>
@@ -2629,21 +4143,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{83BCB134-41DE-47D5-9456-1C60C9867AFA}">
   <dimension ref="A1:J21"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.6640625" customWidth="1"/>
-    <col min="3" max="3" width="27.265625" style="9" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.59765625" customWidth="1"/>
+    <col min="3" max="3" width="27.33203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.6640625" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="40" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="40" customWidth="1"/>
     <col min="9" max="9" width="9" customWidth="1"/>
-    <col min="10" max="10" width="29.1328125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="29.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
@@ -2672,7 +4186,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>72</v>
       </c>
@@ -2702,7 +4216,7 @@
         <v>457 Oak St San Jose, CA, 95101</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>71</v>
       </c>
@@ -2732,7 +4246,7 @@
         <v>203 Birch St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>73</v>
       </c>
@@ -2762,7 +4276,7 @@
         <v>790 Pine St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>74</v>
       </c>
@@ -2792,7 +4306,7 @@
         <v>457 Oak St San Jose, CA, 95101</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>75</v>
       </c>
@@ -2822,7 +4336,7 @@
         <v>459 Oak St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>76</v>
       </c>
@@ -2852,7 +4366,7 @@
         <v>204 Birch St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>77</v>
       </c>
@@ -2882,7 +4396,7 @@
         <v>790 Pine St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>78</v>
       </c>
@@ -2912,7 +4426,7 @@
         <v>204 Birch St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>79</v>
       </c>
@@ -2942,7 +4456,7 @@
         <v>123 Elm St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>80</v>
       </c>
@@ -2972,7 +4486,7 @@
         <v>123 Elm St Los Angeles, CA, 90001</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>81</v>
       </c>
@@ -3002,7 +4516,7 @@
         <v>123 Elm St San Diego, CA, 92101</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
@@ -3032,7 +4546,7 @@
         <v>202 Birch St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>83</v>
       </c>
@@ -3062,7 +4576,7 @@
         <v>204 Birch St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>84</v>
       </c>
@@ -3092,7 +4606,7 @@
         <v>123 Elm St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>85</v>
       </c>
@@ -3122,7 +4636,7 @@
         <v>456 Oak St Chicago, IL, 60601</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>86</v>
       </c>
@@ -3152,7 +4666,7 @@
         <v>203 Birch St Chicago, IL, 60602</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>87</v>
       </c>
@@ -3182,7 +4696,7 @@
         <v>459 Oak St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
@@ -3212,7 +4726,7 @@
         <v>456 Oak St New York, NY, 10001</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>89</v>
       </c>
@@ -3242,7 +4756,7 @@
         <v>459 Oak St Philadelphia, PA, 19101</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>90</v>
       </c>
@@ -3280,23 +4794,23 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A9F197DD-EE87-4022-A4E6-1027B6E64DD6}">
   <dimension ref="A1:N21"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29" style="9" customWidth="1"/>
     <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="11.86328125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="8" width="40" customWidth="1"/>
-    <col min="9" max="9" width="10.59765625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="10.1328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="10.1640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="27.33203125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.6640625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.59765625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
@@ -3338,7 +4852,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>72</v>
       </c>
@@ -3364,7 +4878,7 @@
         <v>11</v>
       </c>
       <c r="I2" t="str" cm="1">
-        <f t="array" ref="I2:J2">_xlfn.TEXTSPLIT(B2," ")</f>
+        <f t="array" ref="I2:J2">_xlfn.TEXTSPLIT(B2, " ")</f>
         <v>Pam</v>
       </c>
       <c r="J2" t="str">
@@ -3383,7 +4897,7 @@
         <v>0123548</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>71</v>
       </c>
@@ -3409,7 +4923,7 @@
         <v>14</v>
       </c>
       <c r="I3" t="str" cm="1">
-        <f t="array" ref="I3:J3">_xlfn.TEXTSPLIT(B3," ")</f>
+        <f t="array" ref="I3:J3">_xlfn.TEXTSPLIT(B3, " ")</f>
         <v>Michael</v>
       </c>
       <c r="J3" t="str">
@@ -3427,7 +4941,7 @@
         <v>0123549</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>73</v>
       </c>
@@ -3453,7 +4967,7 @@
         <v>6</v>
       </c>
       <c r="I4" t="str" cm="1">
-        <f t="array" ref="I4:J4">_xlfn.TEXTSPLIT(B4," ")</f>
+        <f t="array" ref="I4:J4">_xlfn.TEXTSPLIT(B4, " ")</f>
         <v>Kevin</v>
       </c>
       <c r="J4" t="str">
@@ -3471,7 +4985,7 @@
         <v>0123550</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>74</v>
       </c>
@@ -3497,7 +5011,7 @@
         <v>11</v>
       </c>
       <c r="I5" t="str" cm="1">
-        <f t="array" ref="I5:J5">_xlfn.TEXTSPLIT(B5," ")</f>
+        <f t="array" ref="I5:J5">_xlfn.TEXTSPLIT(B5, " ")</f>
         <v>Pam</v>
       </c>
       <c r="J5" t="str">
@@ -3515,7 +5029,7 @@
         <v>0123551</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>75</v>
       </c>
@@ -3541,7 +5055,7 @@
         <v>10</v>
       </c>
       <c r="I6" t="str" cm="1">
-        <f t="array" ref="I6:J6">_xlfn.TEXTSPLIT(B6," ")</f>
+        <f t="array" ref="I6:J6">_xlfn.TEXTSPLIT(B6, " ")</f>
         <v>Jim</v>
       </c>
       <c r="J6" t="str">
@@ -3559,7 +5073,7 @@
         <v>0123552</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>76</v>
       </c>
@@ -3585,7 +5099,7 @@
         <v>15</v>
       </c>
       <c r="I7" t="str" cm="1">
-        <f t="array" ref="I7:J7">_xlfn.TEXTSPLIT(B7," ")</f>
+        <f t="array" ref="I7:J7">_xlfn.TEXTSPLIT(B7, " ")</f>
         <v>Ryan</v>
       </c>
       <c r="J7" t="str">
@@ -3600,7 +5114,7 @@
         <v>0123553</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>77</v>
       </c>
@@ -3626,7 +5140,7 @@
         <v>6</v>
       </c>
       <c r="I8" t="str" cm="1">
-        <f t="array" ref="I8:J8">_xlfn.TEXTSPLIT(B8," ")</f>
+        <f t="array" ref="I8:J8">_xlfn.TEXTSPLIT(B8, " ")</f>
         <v>Kevin</v>
       </c>
       <c r="J8" t="str">
@@ -3641,7 +5155,7 @@
         <v>0123554</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>78</v>
       </c>
@@ -3667,7 +5181,7 @@
         <v>15</v>
       </c>
       <c r="I9" t="str" cm="1">
-        <f t="array" ref="I9:J9">_xlfn.TEXTSPLIT(B9," ")</f>
+        <f t="array" ref="I9:J9">_xlfn.TEXTSPLIT(B9, " ")</f>
         <v>Ryan</v>
       </c>
       <c r="J9" t="str">
@@ -3682,7 +5196,7 @@
         <v>0123555</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>79</v>
       </c>
@@ -3708,7 +5222,7 @@
         <v>18</v>
       </c>
       <c r="I10" t="str" cm="1">
-        <f t="array" ref="I10:J10">_xlfn.TEXTSPLIT(B10," ")</f>
+        <f t="array" ref="I10:J10">_xlfn.TEXTSPLIT(B10, " ")</f>
         <v>Stanley</v>
       </c>
       <c r="J10" t="str">
@@ -3723,7 +5237,7 @@
         <v>0123556</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>80</v>
       </c>
@@ -3749,7 +5263,7 @@
         <v>13</v>
       </c>
       <c r="I11" t="str" cm="1">
-        <f t="array" ref="I11:J11">_xlfn.TEXTSPLIT(B11," ")</f>
+        <f t="array" ref="I11:J11">_xlfn.TEXTSPLIT(B11, " ")</f>
         <v>Angela</v>
       </c>
       <c r="J11" t="str">
@@ -3764,7 +5278,7 @@
         <v>0123557</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>81</v>
       </c>
@@ -3790,7 +5304,7 @@
         <v>17</v>
       </c>
       <c r="I12" t="str" cm="1">
-        <f t="array" ref="I12:J12">_xlfn.TEXTSPLIT(B12," ")</f>
+        <f t="array" ref="I12:J12">_xlfn.TEXTSPLIT(B12, " ")</f>
         <v>Dwight</v>
       </c>
       <c r="J12" t="str">
@@ -3805,7 +5319,7 @@
         <v>0123558</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
@@ -3831,7 +5345,7 @@
         <v>16</v>
       </c>
       <c r="I13" t="str" cm="1">
-        <f t="array" ref="I13:J13">_xlfn.TEXTSPLIT(B13," ")</f>
+        <f t="array" ref="I13:J13">_xlfn.TEXTSPLIT(B13, " ")</f>
         <v>Oscar</v>
       </c>
       <c r="J13" t="str">
@@ -3846,7 +5360,7 @@
         <v>0123559</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>83</v>
       </c>
@@ -3872,7 +5386,7 @@
         <v>15</v>
       </c>
       <c r="I14" t="str" cm="1">
-        <f t="array" ref="I14:J14">_xlfn.TEXTSPLIT(B14," ")</f>
+        <f t="array" ref="I14:J14">_xlfn.TEXTSPLIT(B14, " ")</f>
         <v>Ryan</v>
       </c>
       <c r="J14" t="str">
@@ -3887,7 +5401,7 @@
         <v>0123560</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>84</v>
       </c>
@@ -3913,7 +5427,7 @@
         <v>19</v>
       </c>
       <c r="I15" t="str" cm="1">
-        <f t="array" ref="I15:J15">_xlfn.TEXTSPLIT(B15," ")</f>
+        <f t="array" ref="I15:J15">_xlfn.TEXTSPLIT(B15, " ")</f>
         <v>Phyllis</v>
       </c>
       <c r="J15" t="str">
@@ -3928,7 +5442,7 @@
         <v>0123561</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>85</v>
       </c>
@@ -3954,7 +5468,7 @@
         <v>20</v>
       </c>
       <c r="I16" t="str" cm="1">
-        <f t="array" ref="I16:J16">_xlfn.TEXTSPLIT(B16," ")</f>
+        <f t="array" ref="I16:J16">_xlfn.TEXTSPLIT(B16, " ")</f>
         <v>Meredith</v>
       </c>
       <c r="J16" t="str">
@@ -3969,7 +5483,7 @@
         <v>0123562</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>86</v>
       </c>
@@ -3995,7 +5509,7 @@
         <v>14</v>
       </c>
       <c r="I17" t="str" cm="1">
-        <f t="array" ref="I17:J17">_xlfn.TEXTSPLIT(B17," ")</f>
+        <f t="array" ref="I17:J17">_xlfn.TEXTSPLIT(B17, " ")</f>
         <v>Michael</v>
       </c>
       <c r="J17" t="str">
@@ -4010,7 +5524,7 @@
         <v>0123563</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>87</v>
       </c>
@@ -4036,7 +5550,7 @@
         <v>10</v>
       </c>
       <c r="I18" t="str" cm="1">
-        <f t="array" ref="I18:J18">_xlfn.TEXTSPLIT(B18," ")</f>
+        <f t="array" ref="I18:J18">_xlfn.TEXTSPLIT(B18, " ")</f>
         <v>Jim</v>
       </c>
       <c r="J18" t="str">
@@ -4051,7 +5565,7 @@
         <v>0123564</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
@@ -4077,7 +5591,7 @@
         <v>8</v>
       </c>
       <c r="I19" t="str" cm="1">
-        <f t="array" ref="I19:J19">_xlfn.TEXTSPLIT(B19," ")</f>
+        <f t="array" ref="I19:J19">_xlfn.TEXTSPLIT(B19, " ")</f>
         <v>Kelly</v>
       </c>
       <c r="J19" t="str">
@@ -4092,7 +5606,7 @@
         <v>0123565</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>89</v>
       </c>
@@ -4118,7 +5632,7 @@
         <v>10</v>
       </c>
       <c r="I20" t="str" cm="1">
-        <f t="array" ref="I20:J20">_xlfn.TEXTSPLIT(B20," ")</f>
+        <f t="array" ref="I20:J20">_xlfn.TEXTSPLIT(B20, " ")</f>
         <v>Jim</v>
       </c>
       <c r="J20" t="str">
@@ -4133,7 +5647,7 @@
         <v>0123566</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:14" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>90</v>
       </c>
@@ -4159,7 +5673,7 @@
         <v>10</v>
       </c>
       <c r="I21" t="str" cm="1">
-        <f t="array" ref="I21:J21">_xlfn.TEXTSPLIT(B21," ")</f>
+        <f t="array" ref="I21:J21">_xlfn.TEXTSPLIT(B21, " ")</f>
         <v>Jim</v>
       </c>
       <c r="J21" t="str">
@@ -4182,21 +5696,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E73CB36-69AF-4B27-BCC8-FDB353A4DE72}">
   <dimension ref="A1:L21"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.3984375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14" style="9" customWidth="1"/>
-    <col min="4" max="4" width="16.1328125" customWidth="1"/>
-    <col min="5" max="5" width="26.1328125" customWidth="1"/>
+    <col min="4" max="4" width="16.1640625" customWidth="1"/>
+    <col min="5" max="5" width="26.1640625" customWidth="1"/>
     <col min="6" max="6" width="22" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="37" customWidth="1"/>
     <col min="8" max="8" width="40" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="11.59765625" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="9.1328125" customWidth="1"/>
+    <col min="9" max="9" width="11.6640625" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>69</v>
       </c>
@@ -4227,7 +5741,7 @@
       <c r="K1" s="17"/>
       <c r="L1" s="17"/>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
         <v>72</v>
       </c>
@@ -4265,7 +5779,7 @@
         <v>CA</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
         <v>71</v>
       </c>
@@ -4303,7 +5817,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="5" t="s">
         <v>73</v>
       </c>
@@ -4341,7 +5855,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="5" t="s">
         <v>74</v>
       </c>
@@ -4379,7 +5893,7 @@
         <v>CA</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>75</v>
       </c>
@@ -4417,7 +5931,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="5" t="s">
         <v>76</v>
       </c>
@@ -4455,7 +5969,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="5" t="s">
         <v>77</v>
       </c>
@@ -4493,7 +6007,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
         <v>78</v>
       </c>
@@ -4531,7 +6045,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="5" t="s">
         <v>79</v>
       </c>
@@ -4569,7 +6083,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="5" t="s">
         <v>80</v>
       </c>
@@ -4607,7 +6121,7 @@
         <v>CA</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="5" t="s">
         <v>81</v>
       </c>
@@ -4645,7 +6159,7 @@
         <v>CA</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="5" t="s">
         <v>82</v>
       </c>
@@ -4683,7 +6197,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="5" t="s">
         <v>83</v>
       </c>
@@ -4721,7 +6235,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="5" t="s">
         <v>84</v>
       </c>
@@ -4759,7 +6273,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="5" t="s">
         <v>85</v>
       </c>
@@ -4797,7 +6311,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="5" t="s">
         <v>86</v>
       </c>
@@ -4835,7 +6349,7 @@
         <v>IL</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="5" t="s">
         <v>87</v>
       </c>
@@ -4873,7 +6387,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="5" t="s">
         <v>88</v>
       </c>
@@ -4911,7 +6425,7 @@
         <v>NY</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="5" t="s">
         <v>89</v>
       </c>
@@ -4949,7 +6463,7 @@
         <v>PA</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="14.65" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="21" spans="1:12" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>90</v>
       </c>
@@ -4997,31 +6511,31 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85789AE4-586B-4DA1-B069-1172780CDADC}">
-  <dimension ref="A2:BW25"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A2:BW58"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="24.3984375" customWidth="1"/>
+    <col min="1" max="1" width="24.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A2" s="15" t="s">
         <v>94</v>
       </c>
       <c r="B2" s="16"/>
     </row>
-    <row r="3" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A3" t="str">
         <f>_xlfn.TEXTJOIN(", ",TRUE,Data!H2:H21)</f>
         <v>Kafka, DataBricks, Spark, Python, GCP, Power BI, GCP, Airflow, Hadoop, R, Azure, Java, SQL, DataBricks, Kafka, DataBricks, Spark, Python, GCP, DataBricks, Hadoop, Java, Snowflake, Airflow, DataBricks, Azure, Java, SQL, DataBricks, Snowflake, Airflow, DataBricks, Scala, Azure, R, Kafka, Snowflake, Excel, Scala, Excel, Power BI, R, Scala, R, Hadoop, Power BI, SQL, Snowflake, Airflow, DataBricks, Java, Scala, R, DataBricks, Azure, Scala, Power BI, GCP, Airflow, Hadoop, R, DataBricks, Hadoop, Java, Snowflake, Power BI, Tableau, Airflow, SQL, DataBricks, Hadoop, Java, DataBricks, Hadoop, Java</v>
       </c>
     </row>
-    <row r="5" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A5" s="15" t="s">
         <v>67</v>
       </c>
       <c r="B5" s="16"/>
     </row>
-    <row r="6" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A6" t="str" cm="1">
         <f t="array" ref="A6:BW6">_xlfn.TEXTSPLIT(A3,", ")</f>
         <v>Kafka</v>
@@ -5249,7 +6763,7 @@
         <v>Java</v>
       </c>
     </row>
-    <row r="8" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
         <v>68</v>
       </c>
@@ -5261,7 +6775,7 @@
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
     </row>
-    <row r="9" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="str" cm="1">
         <f t="array" ref="A9:A25">_xlfn.UNIQUE(TRANSPOSE(6:6))</f>
         <v>Kafka</v>
@@ -5271,7 +6785,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="str">
         <v>DataBricks</v>
       </c>
@@ -5280,7 +6794,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="str">
         <v>Spark</v>
       </c>
@@ -5289,7 +6803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="str">
         <v>Python</v>
       </c>
@@ -5298,7 +6812,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="str">
         <v>GCP</v>
       </c>
@@ -5307,7 +6821,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="str">
         <v>Power BI</v>
       </c>
@@ -5316,7 +6830,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="str">
         <v>Airflow</v>
       </c>
@@ -5325,7 +6839,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:75" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:75" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="str">
         <v>Hadoop</v>
       </c>
@@ -5334,7 +6848,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="str">
         <v>R</v>
       </c>
@@ -5343,7 +6857,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="str">
         <v>Azure</v>
       </c>
@@ -5352,7 +6866,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="str">
         <v>Java</v>
       </c>
@@ -5361,7 +6875,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="str">
         <v>SQL</v>
       </c>
@@ -5370,7 +6884,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="str">
         <v>Snowflake</v>
       </c>
@@ -5379,7 +6893,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="str">
         <v>Scala</v>
       </c>
@@ -5388,7 +6902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="str">
         <v>Excel</v>
       </c>
@@ -5397,7 +6911,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="str">
         <v>Tableau</v>
       </c>
@@ -5406,12 +6920,442 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>0</v>
       </c>
       <c r="B25" s="1">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="str">
+        <f>_xlfn.TEXTJOIN(", ",TRUE,Data!H2:H21)</f>
+        <v>Kafka, DataBricks, Spark, Python, GCP, Power BI, GCP, Airflow, Hadoop, R, Azure, Java, SQL, DataBricks, Kafka, DataBricks, Spark, Python, GCP, DataBricks, Hadoop, Java, Snowflake, Airflow, DataBricks, Azure, Java, SQL, DataBricks, Snowflake, Airflow, DataBricks, Scala, Azure, R, Kafka, Snowflake, Excel, Scala, Excel, Power BI, R, Scala, R, Hadoop, Power BI, SQL, Snowflake, Airflow, DataBricks, Java, Scala, R, DataBricks, Azure, Scala, Power BI, GCP, Airflow, Hadoop, R, DataBricks, Hadoop, Java, Snowflake, Power BI, Tableau, Airflow, SQL, DataBricks, Hadoop, Java, DataBricks, Hadoop, Java</v>
+      </c>
+    </row>
+    <row r="33" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A33" t="str" cm="1">
+        <f t="array" ref="A33:BW33">_xlfn.TEXTSPLIT(A31,", ")</f>
+        <v>Kafka</v>
+      </c>
+      <c r="B33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Spark</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Python</v>
+      </c>
+      <c r="E33" t="str">
+        <v>GCP</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="G33" t="str">
+        <v>GCP</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="J33" t="str">
+        <v>R</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Azure</v>
+      </c>
+      <c r="L33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="M33" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="N33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Kafka</v>
+      </c>
+      <c r="P33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>Spark</v>
+      </c>
+      <c r="R33" t="str">
+        <v>Python</v>
+      </c>
+      <c r="S33" t="str">
+        <v>GCP</v>
+      </c>
+      <c r="T33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="U33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="V33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="W33" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="X33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="Y33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="Z33" t="str">
+        <v>Azure</v>
+      </c>
+      <c r="AA33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="AB33" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="AC33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="AD33" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="AE33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="AF33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="AG33" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="AH33" t="str">
+        <v>Azure</v>
+      </c>
+      <c r="AI33" t="str">
+        <v>R</v>
+      </c>
+      <c r="AJ33" t="str">
+        <v>Kafka</v>
+      </c>
+      <c r="AK33" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="AL33" t="str">
+        <v>Excel</v>
+      </c>
+      <c r="AM33" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="AN33" t="str">
+        <v>Excel</v>
+      </c>
+      <c r="AO33" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="AP33" t="str">
+        <v>R</v>
+      </c>
+      <c r="AQ33" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="AR33" t="str">
+        <v>R</v>
+      </c>
+      <c r="AS33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="AT33" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="AU33" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="AV33" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="AW33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="AX33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="AY33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="AZ33" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="BA33" t="str">
+        <v>R</v>
+      </c>
+      <c r="BB33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="BC33" t="str">
+        <v>Azure</v>
+      </c>
+      <c r="BD33" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="BE33" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="BF33" t="str">
+        <v>GCP</v>
+      </c>
+      <c r="BG33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="BH33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="BI33" t="str">
+        <v>R</v>
+      </c>
+      <c r="BJ33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="BK33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="BL33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="BM33" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="BN33" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="BO33" t="str">
+        <v>Tableau</v>
+      </c>
+      <c r="BP33" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="BQ33" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="BR33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="BS33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="BT33" t="str">
+        <v>Java</v>
+      </c>
+      <c r="BU33" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="BV33" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="BW33" t="str">
+        <v>Java</v>
+      </c>
+    </row>
+    <row r="35" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A35" t="str" cm="1">
+        <f t="array" ref="A35:A51">_xlfn.UNIQUE(TRANSPOSE(33:33))</f>
+        <v>Kafka</v>
+      </c>
+      <c r="B35">
+        <f>COUNTIF($33:$33,A35)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A36" t="str">
+        <v>DataBricks</v>
+      </c>
+      <c r="B36">
+        <f t="shared" ref="B36:B58" si="1">COUNTIF($33:$33,A36)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A37" t="str">
+        <v>Spark</v>
+      </c>
+      <c r="B37">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A38" t="str">
+        <v>Python</v>
+      </c>
+      <c r="B38">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A39" t="str">
+        <v>GCP</v>
+      </c>
+      <c r="B39">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A40" t="str">
+        <v>Power BI</v>
+      </c>
+      <c r="B40">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A41" t="str">
+        <v>Airflow</v>
+      </c>
+      <c r="B41">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="42" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A42" t="str">
+        <v>Hadoop</v>
+      </c>
+      <c r="B42">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A43" t="str">
+        <v>R</v>
+      </c>
+      <c r="B43">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="44" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A44" t="str">
+        <v>Azure</v>
+      </c>
+      <c r="B44">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="45" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A45" t="str">
+        <v>Java</v>
+      </c>
+      <c r="B45">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A46" t="str">
+        <v>SQL</v>
+      </c>
+      <c r="B46">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A47" t="str">
+        <v>Snowflake</v>
+      </c>
+      <c r="B47">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="48" spans="1:75" x14ac:dyDescent="0.2">
+      <c r="A48" t="str">
+        <v>Scala</v>
+      </c>
+      <c r="B48">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" t="str">
+        <v>Excel</v>
+      </c>
+      <c r="B49">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" t="str">
+        <v>Tableau</v>
+      </c>
+      <c r="B50">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>0</v>
+      </c>
+      <c r="B51">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B52">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B53">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B54">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B55">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B56">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B57">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B58">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>